<commit_message>
Add Morris interaction and stability figures
</commit_message>
<xml_diff>
--- a/示例输入/ExcelInterface-master/Example input/SingleLayerLoam2D/sensitivity_runs/formal_r300_workers16_timeout300/figures/morris_sensitivity_without_slow_tables.xlsx
+++ b/示例输入/ExcelInterface-master/Example input/SingleLayerLoam2D/sensitivity_runs/formal_r300_workers16_timeout300/figures/morris_sensitivity_without_slow_tables.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Morris_indices'!$A$1:$J$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Normalized_by_output'!$A$1:$J$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Normalized_summary'!$A$1:$G$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Method_notes'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Method_notes'!$A$1:$B$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8290,7 +8290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8348,41 +8348,65 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Figure2</t>
+          <t>Figure1</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>The plotted ranking figure shows the top 6 parameters for each output metric by mu_star.</t>
+          <t>The Morris mu_star-sigma plane is exported to assess parameter importance together with nonlinearity or interaction effects.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Figure5</t>
+          <t>Figure2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Mean normalized sensitivity is derived by dividing mu_star by the maximum mu_star within each output metric, then averaging by parameter.</t>
+          <t>The plotted ranking figure shows the top 6 parameters for each output metric by mu_star.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>Figure5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Mean normalized sensitivity is derived by dividing mu_star by the maximum mu_star within each output metric, then averaging by parameter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Figure6</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>The sigma/mu_star ratio is plotted for the top 6 parameters of each output metric to indicate effect stability among important parameters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>Sigma</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>sigma is retained in the complete Morris table for assessing nonlinearity or interaction effects.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>